<commit_message>
Update frontend and fix normalization
</commit_message>
<xml_diff>
--- a/outputs/ranked_candidates.xlsx
+++ b/outputs/ranked_candidates.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0001218</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -452,511 +452,511 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AI Specialist with 6.4 yrs; 4 AI core skills; response rate 0.82.</t>
+          <t>Senior Machine Learning Engineer with 7.2 yrs; 9 AI core skills; response rate 0.61.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0092278</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9336</v>
+        <v>0.9947</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer with 6.8 yrs; 7 AI core skills; response rate 0.07.</t>
+          <t>Staff Machine Learning Engineer with 7.0 yrs; 9 AI core skills; response rate 0.95.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0039754</t>
+          <t>CAND_0081846</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8527</v>
+        <v>0.9918</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist with 16.2 yrs; 8 AI core skills; response rate 0.81.</t>
+          <t>Lead AI Engineer with 6.7 yrs; 10 AI core skills; response rate 0.73.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0086022</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8282</v>
+        <v>0.9905</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer with 7.2 yrs; 9 AI core skills; response rate 0.61.</t>
+          <t>Senior Applied Scientist with 5.3 yrs; 8 AI core skills; response rate 0.55.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0046064</t>
+          <t>CAND_0005509</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7567</v>
+        <v>0.978</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer with 8.9 yrs; 6 AI core skills; response rate 0.78.</t>
+          <t>Data Scientist with 6.0 yrs; 2 AI core skills; response rate 0.40.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0044262</t>
+          <t>CAND_0079387</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>0.7311</v>
+        <v>0.978</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Data Scientist with 6.9 yrs; 4 AI core skills; response rate 0.73.</t>
+          <t>AI Engineer with 6.9 yrs; 5 AI core skills; response rate 0.81.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CAND_0058412</t>
+          <t>CAND_0039754</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7183</v>
+        <v>0.9766</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.6 yrs; 3 AI core skills; response rate 0.43.</t>
+          <t>Senior Applied Scientist with 16.2 yrs; 8 AI core skills; response rate 0.81.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CAND_0088025</t>
+          <t>CAND_0046064</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7161999999999999</v>
+        <v>0.9727</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer with 8.6 yrs; 9 AI core skills; response rate 0.83.</t>
+          <t>Senior NLP Engineer with 8.9 yrs; 6 AI core skills; response rate 0.78.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CAND_0030953</t>
+          <t>CAND_0080534</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>0.7089</v>
+        <v>0.9726</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Search Engineer with 7.8 yrs; 5 AI core skills; response rate 0.63.</t>
+          <t>ML Engineer with 3.8 yrs; 5 AI core skills; response rate 0.91.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.6951000000000001</v>
+        <v>0.9567</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer with 7.0 yrs; 9 AI core skills; response rate 0.95.</t>
+          <t>Senior Machine Learning Engineer with 6.1 yrs; 5 AI core skills; response rate 0.88.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CAND_0071974</t>
+          <t>CAND_0065786</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>0.6853</v>
+        <v>0.9529</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Senior AI Engineer with 7.8 yrs; 9 AI core skills; response rate 0.76.</t>
+          <t>AI Specialist with 4.9 yrs; 5 AI core skills; response rate 0.89.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CAND_0041611</t>
+          <t>CAND_0088025</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>0.6834</v>
+        <v>0.9523</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer with 6.4 yrs; 7 AI core skills; response rate 0.07.</t>
+          <t>Staff Machine Learning Engineer with 8.6 yrs; 9 AI core skills; response rate 0.83.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CAND_0025882</t>
+          <t>CAND_0071974</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.9502</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 5.6 yrs; 6 AI core skills; response rate 0.79.</t>
+          <t>Senior AI Engineer with 7.8 yrs; 9 AI core skills; response rate 0.76.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CAND_0069638</t>
+          <t>CAND_0097176</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>0.6786</v>
+        <v>0.95</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 6.2 yrs; 4 AI core skills; response rate 0.64.</t>
+          <t>ML Engineer with 5.9 yrs; 2 AI core skills; response rate 0.76.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CAND_0067717</t>
+          <t>CAND_0091580</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>0.6771</v>
+        <v>0.9477</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AI Specialist with 6.9 yrs; 4 AI core skills; response rate 0.39.</t>
+          <t>Data Scientist with 5.5 yrs; 4 AI core skills; response rate 0.25.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CAND_0047521</t>
+          <t>CAND_0055992</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>0.6753</v>
+        <v>0.9451000000000001</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 4.4 yrs; 5 AI core skills; response rate 0.83.</t>
+          <t>AI Engineer with 16.9 yrs; 8 AI core skills; response rate 0.72.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAND_0093883</t>
+          <t>CAND_0043304</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>0.6751</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 5.0 yrs; 6 AI core skills; response rate 0.56.</t>
+          <t>Junior ML Engineer with 6.5 yrs; 2 AI core skills; response rate 0.75.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CAND_0055905</t>
+          <t>CAND_0010149</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>0.6694</v>
+        <v>0.9374</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer with 8.1 yrs; 5 AI core skills; response rate 0.87.</t>
+          <t>ML Engineer with 6.9 yrs; 4 AI core skills; response rate 0.82.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CAND_0009691</t>
+          <t>CAND_0052195</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>0.663</v>
+        <v>0.9364</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 6.2 yrs; 5 AI core skills; response rate 0.64.</t>
+          <t>Computer Vision Engineer with 6.3 yrs; 2 AI core skills; response rate 0.69.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAND_0021410</t>
+          <t>CAND_0048166</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>0.6536999999999999</v>
+        <v>0.9362</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 4.0 yrs; 4 AI core skills; response rate 0.80.</t>
+          <t>ML Engineer with 5.2 yrs; 3 AI core skills; response rate 0.48.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CAND_0010149</t>
+          <t>CAND_0025882</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>0.648</v>
+        <v>0.9356</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ML Engineer with 6.9 yrs; 4 AI core skills; response rate 0.82.</t>
+          <t>Senior Software Engineer (ML) with 5.6 yrs; 6 AI core skills; response rate 0.79.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CAND_0046924</t>
+          <t>CAND_0001494</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>0.6467000000000001</v>
+        <v>0.9322</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 6.3 yrs; 8 AI core skills; response rate 0.61.</t>
+          <t>Data Scientist with 6.4 yrs; 4 AI core skills; response rate 0.30.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CAND_0067643</t>
+          <t>CAND_0001930</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>0.6443</v>
+        <v>0.9298999999999999</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 6.0 yrs; 4 AI core skills; response rate 0.49.</t>
+          <t>Senior Software Engineer (ML) with 6.9 yrs; 1 AI core skills; response rate 0.65.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CAND_0001930</t>
+          <t>CAND_0078262</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>0.6417</v>
+        <v>0.9248</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.9 yrs; 1 AI core skills; response rate 0.65.</t>
+          <t>ML Engineer with 4.9 yrs; 4 AI core skills; response rate 0.39.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CAND_0069771</t>
+          <t>CAND_0008425</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>0.6412</v>
+        <v>0.9245</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.7 yrs; 7 AI core skills; response rate 0.36.</t>
+          <t>Senior NLP Engineer with 7.8 yrs; 5 AI core skills; response rate 0.66.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CAND_0065786</t>
+          <t>CAND_0023215</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>0.6389</v>
+        <v>0.9242</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>AI Specialist with 4.9 yrs; 5 AI core skills; response rate 0.89.</t>
+          <t>Junior ML Engineer with 4.4 yrs; 3 AI core skills; response rate 0.43.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CAND_0061479</t>
+          <t>CAND_0006538</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>0.6375</v>
+        <v>0.9238</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ML Engineer with 5.0 yrs; 4 AI core skills; response rate 0.81.</t>
+          <t>AI Specialist with 5.7 yrs; 5 AI core skills; response rate 0.86.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CAND_0086028</t>
+          <t>CAND_0090300</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>0.637</v>
+        <v>0.9238</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 6.2 yrs; 3 AI core skills; response rate 0.29.</t>
+          <t>AI Research Engineer with 5.3 yrs; 3 AI core skills; response rate 0.94.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CAND_0017648</t>
+          <t>CAND_0049615</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>0.6349</v>
+        <v>0.9232</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>AI Specialist with 4.0 yrs; 3 AI core skills; response rate 0.62.</t>
+          <t>ML Engineer with 5.1 yrs; 3 AI core skills; response rate 0.28.</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>0.6293</v>
+        <v>0.9232</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -981,1260 +981,1260 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CAND_0077552</t>
+          <t>CAND_0069248</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>0.6289</v>
+        <v>0.9226</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 3.4 yrs; 3 AI core skills; response rate 0.54.</t>
+          <t>AI Research Engineer with 5.4 yrs; 2 AI core skills; response rate 0.75.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CAND_0055139</t>
+          <t>CAND_0067866</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>0.6286</v>
+        <v>0.9204</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ML Engineer with 6.9 yrs; 4 AI core skills; response rate 0.25.</t>
+          <t>Senior Software Engineer (ML) with 6.4 yrs; 3 AI core skills; response rate 0.79.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CAND_0009236</t>
+          <t>CAND_0013613</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>0.6281</v>
+        <v>0.9193</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>AI Specialist with 6.3 yrs; 4 AI core skills; response rate 0.32.</t>
+          <t>Machine Learning Engineer with 4.7 yrs; 4 AI core skills; response rate 0.73.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CAND_0097896</t>
+          <t>CAND_0005649</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>0.6277</v>
+        <v>0.9188</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 4.8 yrs; 6 AI core skills; response rate 0.65.</t>
+          <t>Senior Data Scientist with 7.4 yrs; 7 AI core skills; response rate 0.57.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CAND_0008425</t>
+          <t>CAND_0000031</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>0.6231</v>
+        <v>0.915</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer with 7.8 yrs; 5 AI core skills; response rate 0.66.</t>
+          <t>Recommendation Systems Engineer with 6.0 yrs; 7 AI core skills; response rate 0.91.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAND_0056262</t>
+          <t>CAND_0055905</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>0.6191</v>
+        <v>0.9146</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 6.0 yrs; 3 AI core skills; response rate 0.29.</t>
+          <t>Senior Machine Learning Engineer with 8.1 yrs; 5 AI core skills; response rate 0.87.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CAND_0087630</t>
+          <t>CAND_0002025</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>0.6167</v>
+        <v>0.9146</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>AI Engineer with 7.2 yrs; 6 AI core skills; response rate 0.45.</t>
+          <t>Senior AI Engineer with 5.9 yrs; 7 AI core skills; response rate 0.80.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CAND_0033861</t>
+          <t>CAND_0069905</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>0.6156</v>
+        <v>0.9134</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer with 8.0 yrs; 10 AI core skills; response rate 0.16.</t>
+          <t>Applied ML Engineer with 6.6 yrs; 4 AI core skills; response rate 0.78.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAND_0081846</t>
+          <t>CAND_0068932</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>0.6084000000000001</v>
+        <v>0.9122</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Lead AI Engineer with 6.7 yrs; 10 AI core skills; response rate 0.73.</t>
+          <t>ML Engineer with 5.2 yrs; 5 AI core skills; response rate 0.82.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAND_0049615</t>
+          <t>CAND_0064130</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>0.6014</v>
+        <v>0.9121</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>ML Engineer with 5.1 yrs; 3 AI core skills; response rate 0.28.</t>
+          <t>AI Research Engineer with 6.7 yrs; 3 AI core skills; response rate 0.67.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAND_0060072</t>
+          <t>CAND_0032955</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>0.5974</v>
+        <v>0.9121</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer with 5.7 yrs; 8 AI core skills; response rate 0.10.</t>
+          <t>Computer Vision Engineer with 5.2 yrs; 3 AI core skills; response rate 0.26.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CAND_0001494</t>
+          <t>CAND_0072232</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>0.5921999999999999</v>
+        <v>0.9106</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Data Scientist with 6.4 yrs; 4 AI core skills; response rate 0.30.</t>
+          <t>ML Engineer with 4.0 yrs; 3 AI core skills; response rate 0.58.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CAND_0054703</t>
+          <t>CAND_0061339</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>0.5919</v>
+        <v>0.9101</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 6.8 yrs; 3 AI core skills; response rate 0.41.</t>
+          <t>Search Engineer with 4.2 yrs; 7 AI core skills; response rate 0.90.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CAND_0033749</t>
+          <t>CAND_0069638</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>0.5915</v>
+        <v>0.9101</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 4.7 yrs; 8 AI core skills; response rate 0.78.</t>
+          <t>Computer Vision Engineer with 6.2 yrs; 4 AI core skills; response rate 0.64.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CAND_0018653</t>
+          <t>CAND_0087630</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>0.5911999999999999</v>
+        <v>0.9093</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ML Engineer with 6.5 yrs; 5 AI core skills; response rate 0.72.</t>
+          <t>AI Engineer with 7.2 yrs; 6 AI core skills; response rate 0.45.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CAND_0051486</t>
+          <t>CAND_0060315</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>0.591</v>
+        <v>0.9081</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>AI Specialist with 5.9 yrs; 6 AI core skills; response rate 0.60.</t>
+          <t>Senior Software Engineer (ML) with 5.4 yrs; 5 AI core skills; response rate 0.63.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CAND_0093185</t>
+          <t>CAND_0050876</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>0.5908</v>
+        <v>0.9077</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 4.1 yrs; 5 AI core skills; response rate 0.60.</t>
+          <t>Applied ML Engineer with 6.0 yrs; 6 AI core skills; response rate 0.67.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CAND_0058882</t>
+          <t>CAND_0012837</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>0.5905</v>
+        <v>0.9071</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 3.6 yrs; 7 AI core skills; response rate 0.42.</t>
+          <t>Junior ML Engineer with 6.4 yrs; 5 AI core skills; response rate 0.81.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAND_0048166</t>
+          <t>CAND_0044855</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>0.5861</v>
+        <v>0.9069</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ML Engineer with 5.2 yrs; 3 AI core skills; response rate 0.48.</t>
+          <t>Senior Data Scientist with 6.6 yrs; 6 AI core skills; response rate 0.57.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAND_0078262</t>
+          <t>CAND_0060054</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>0.5859</v>
+        <v>0.9065</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ML Engineer with 4.9 yrs; 4 AI core skills; response rate 0.39.</t>
+          <t>AI Engineer with 6.4 yrs; 6 AI core skills; response rate 0.86.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CAND_0013393</t>
+          <t>CAND_0077296</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>0.5855</v>
+        <v>0.9059</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ML Engineer with 5.3 yrs; 7 AI core skills; response rate 0.33.</t>
+          <t>Computer Vision Engineer with 5.8 yrs; 3 AI core skills; response rate 0.50.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CAND_0008978</t>
+          <t>CAND_0008517</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.9053</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 6.7 yrs; 7 AI core skills; response rate 0.29.</t>
+          <t>AI Research Engineer with 5.6 yrs; 4 AI core skills; response rate 0.80.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CAND_0006538</t>
+          <t>CAND_0018925</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>0.5828</v>
+        <v>0.9046</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>AI Specialist with 5.7 yrs; 5 AI core skills; response rate 0.86.</t>
+          <t>AI Research Engineer with 5.8 yrs; 3 AI core skills; response rate 0.45.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAND_0091580</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>0.58</v>
+        <v>0.9034</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Data Scientist with 5.5 yrs; 4 AI core skills; response rate 0.25.</t>
+          <t>Senior NLP Engineer with 7.8 yrs; 8 AI core skills; response rate 0.89.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAND_0005509</t>
+          <t>CAND_0081321</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>0.5773</v>
+        <v>0.9033</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Data Scientist with 6.0 yrs; 2 AI core skills; response rate 0.40.</t>
+          <t>Senior Software Engineer (ML) with 5.3 yrs; 4 AI core skills; response rate 0.47.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CAND_0072232</t>
+          <t>CAND_0054703</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>0.5672</v>
+        <v>0.9026999999999999</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ML Engineer with 4.0 yrs; 3 AI core skills; response rate 0.58.</t>
+          <t>Computer Vision Engineer with 6.8 yrs; 3 AI core skills; response rate 0.41.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CAND_0082913</t>
+          <t>CAND_0039383</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>0.5669</v>
+        <v>0.9019</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 5.5 yrs; 7 AI core skills; response rate 0.73.</t>
+          <t>Applied ML Engineer with 7.1 yrs; 5 AI core skills; response rate 0.61.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAND_0066309</t>
+          <t>CAND_0009691</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.9015</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 5.3 yrs; 6 AI core skills; response rate 0.56.</t>
+          <t>Applied ML Engineer with 6.2 yrs; 5 AI core skills; response rate 0.64.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CAND_0008202</t>
+          <t>CAND_0086151</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>0.5567</v>
+        <v>0.9015</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 5.7 yrs; 7 AI core skills; response rate 0.50.</t>
+          <t>Recommendation Systems Engineer with 7.7 yrs; 5 AI core skills; response rate 0.52.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CAND_0055992</t>
+          <t>CAND_0073883</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>0.5552</v>
+        <v>0.9009</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>AI Engineer with 16.9 yrs; 8 AI core skills; response rate 0.72.</t>
+          <t>AI Specialist with 5.3 yrs; 4 AI core skills; response rate 0.92.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAND_0073917</t>
+          <t>CAND_0070525</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>0.5545</v>
+        <v>0.9008</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Data Scientist with 5.8 yrs; 4 AI core skills; response rate 0.46.</t>
+          <t>Senior Software Engineer (ML) with 5.4 yrs; 2 AI core skills; response rate 0.93.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAND_0062772</t>
+          <t>CAND_0033179</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>0.5514</v>
+        <v>0.8989</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.6 yrs; 5 AI core skills; response rate 0.86.</t>
+          <t>AI Research Engineer with 6.9 yrs; 6 AI core skills; response rate 0.84.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CAND_0094759</t>
+          <t>CAND_0021410</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>0.5513</v>
+        <v>0.8979</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Lead AI Engineer with 8.6 yrs; 8 AI core skills; response rate 0.11.</t>
+          <t>Junior ML Engineer with 4.0 yrs; 4 AI core skills; response rate 0.80.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CAND_0013988</t>
+          <t>CAND_0002120</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>0.5482</v>
+        <v>0.8959</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 5.4 yrs; 3 AI core skills; response rate 0.29.</t>
+          <t>ML Engineer with 6.5 yrs; 5 AI core skills; response rate 0.72.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CAND_0016678</t>
+          <t>CAND_0044262</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>0.5479000000000001</v>
+        <v>0.8952</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 6.8 yrs; 2 AI core skills; response rate 0.57.</t>
+          <t>Data Scientist with 6.9 yrs; 4 AI core skills; response rate 0.73.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAND_0081778</t>
+          <t>CAND_0077552</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>0.5445</v>
+        <v>0.8946</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Data Scientist with 6.4 yrs; 1 AI core skills; response rate 0.52.</t>
+          <t>Senior Software Engineer (ML) with 3.4 yrs; 3 AI core skills; response rate 0.54.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAND_0090300</t>
+          <t>CAND_0047521</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>0.5426</v>
+        <v>0.8937</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 5.3 yrs; 3 AI core skills; response rate 0.94.</t>
+          <t>Junior ML Engineer with 4.4 yrs; 5 AI core skills; response rate 0.83.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CAND_0018925</t>
+          <t>CAND_0017960</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>0.5424</v>
+        <v>0.8932</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 5.8 yrs; 3 AI core skills; response rate 0.45.</t>
+          <t>Recommendation Systems Engineer with 7.7 yrs; 2 AI core skills; response rate 0.72.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAND_0074123</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>0.5422</v>
+        <v>0.8919</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Data Scientist with 6.9 yrs; 5 AI core skills; response rate 0.38.</t>
+          <t>Recommendation Systems Engineer with 8.0 yrs; 8 AI core skills; response rate 0.77.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAND_0010770</t>
+          <t>CAND_0003557</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>0.5421</v>
+        <v>0.8911</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer with 15.2 yrs; 7 AI core skills; response rate 0.73.</t>
+          <t>ML Engineer with 6.8 yrs; 4 AI core skills; response rate 0.47.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CAND_0049771</t>
+          <t>CAND_0074123</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>0.5417</v>
+        <v>0.8903</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 5.0 yrs; 3 AI core skills; response rate 0.81.</t>
+          <t>Data Scientist with 6.9 yrs; 5 AI core skills; response rate 0.38.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAND_0033911</t>
+          <t>CAND_0013393</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>0.5417</v>
+        <v>0.8892</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Data Scientist with 6.9 yrs; 6 AI core skills; response rate 0.76.</t>
+          <t>ML Engineer with 5.3 yrs; 7 AI core skills; response rate 0.33.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CAND_0097176</t>
+          <t>CAND_0037160</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>0.5397999999999999</v>
+        <v>0.8881</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>ML Engineer with 5.9 yrs; 2 AI core skills; response rate 0.76.</t>
+          <t>Data Scientist with 6.0 yrs; 6 AI core skills; response rate 0.74.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CAND_0023215</t>
+          <t>CAND_0028422</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>0.5395</v>
+        <v>0.8868</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Junior ML Engineer with 4.4 yrs; 3 AI core skills; response rate 0.43.</t>
+          <t>Junior ML Engineer with 5.5 yrs; 7 AI core skills; response rate 0.76.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAND_0078669</t>
+          <t>CAND_0082913</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>0.5356</v>
+        <v>0.8865</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>ML Engineer with 6.3 yrs; 5 AI core skills; response rate 0.49.</t>
+          <t>Senior Software Engineer (ML) with 5.5 yrs; 7 AI core skills; response rate 0.73.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAND_0005260</t>
+          <t>CAND_0011327</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>0.5355</v>
+        <v>0.886</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer with 5.2 yrs; 6 AI core skills; response rate 0.86.</t>
+          <t>AI Research Engineer with 6.3 yrs; 3 AI core skills; response rate 0.79.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAND_0003756</t>
+          <t>CAND_0016170</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>0.5353</v>
+        <v>0.8856000000000001</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 6.5 yrs; 3 AI core skills; response rate 0.38.</t>
+          <t>AI Research Engineer with 6.8 yrs; 2 AI core skills; response rate 0.52.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CAND_0049217</t>
+          <t>CAND_0067643</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>0.5347</v>
+        <v>0.884</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 6.0 yrs; 3 AI core skills; response rate 0.87.</t>
+          <t>AI Research Engineer with 6.0 yrs; 4 AI core skills; response rate 0.49.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAND_0080534</t>
+          <t>CAND_0058300</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>0.5339</v>
+        <v>0.8838</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>ML Engineer with 3.8 yrs; 5 AI core skills; response rate 0.91.</t>
+          <t>AI Research Engineer with 4.5 yrs; 4 AI core skills; response rate 0.52.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CAND_0074621</t>
+          <t>CAND_0040178</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>0.5327</v>
+        <v>0.8836000000000001</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Data Scientist with 5.2 yrs; 4 AI core skills; response rate 0.74.</t>
+          <t>ML Engineer with 5.0 yrs; 5 AI core skills; response rate 0.55.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CAND_0080344</t>
+          <t>CAND_0032089</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>0.5327</v>
+        <v>0.8836000000000001</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 4.9 yrs; 4 AI core skills; response rate 0.70.</t>
+          <t>ML Engineer with 6.6 yrs; 3 AI core skills; response rate 0.54.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CAND_0002120</t>
+          <t>CAND_0059795</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>0.5303</v>
+        <v>0.882</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ML Engineer with 6.5 yrs; 5 AI core skills; response rate 0.72.</t>
+          <t>Senior Software Engineer (ML) with 5.6 yrs; 1 AI core skills; response rate 0.75.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CAND_0014858</t>
+          <t>CAND_0069771</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>0.5296999999999999</v>
+        <v>0.8816000000000001</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 4.9 yrs; 4 AI core skills; response rate 0.30.</t>
+          <t>Junior ML Engineer with 5.7 yrs; 7 AI core skills; response rate 0.36.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAND_0086062</t>
+          <t>CAND_0033987</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>0.5291</v>
+        <v>0.8811</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>ML Engineer with 4.1 yrs; 3 AI core skills; response rate 0.51.</t>
+          <t>ML Engineer with 6.8 yrs; 4 AI core skills; response rate 0.71.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAND_0060054</t>
+          <t>CAND_0083852</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>0.5269</v>
+        <v>0.8788</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>AI Engineer with 6.4 yrs; 6 AI core skills; response rate 0.86.</t>
+          <t>Data Scientist with 6.0 yrs; 6 AI core skills; response rate 0.85.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAND_0057563</t>
+          <t>CAND_0062772</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>0.5269</v>
+        <v>0.8781</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>NLP Engineer with 6.8 yrs; 5 AI core skills; response rate 0.83.</t>
+          <t>Senior Software Engineer (ML) with 6.6 yrs; 5 AI core skills; response rate 0.86.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CAND_0079387</t>
+          <t>CAND_0017648</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>0.5247000000000001</v>
+        <v>0.878</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>AI Engineer with 6.9 yrs; 5 AI core skills; response rate 0.81.</t>
+          <t>AI Specialist with 4.0 yrs; 3 AI core skills; response rate 0.62.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CAND_0069248</t>
+          <t>CAND_0093883</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>0.524</v>
+        <v>0.8773</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 5.4 yrs; 2 AI core skills; response rate 0.75.</t>
+          <t>AI Research Engineer with 5.0 yrs; 6 AI core skills; response rate 0.56.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CAND_0003557</t>
+          <t>CAND_0026716</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>0.5238</v>
+        <v>0.8771</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>ML Engineer with 6.8 yrs; 4 AI core skills; response rate 0.47.</t>
+          <t>Computer Vision Engineer with 5.6 yrs; 5 AI core skills; response rate 0.82.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CAND_0026610</t>
+          <t>CAND_0078002</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>0.5223</v>
+        <v>0.8766</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 6.4 yrs; 1 AI core skills; response rate 0.67.</t>
+          <t>Machine Learning Engineer with 6.3 yrs; 4 AI core skills; response rate 0.86.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CAND_0044855</t>
+          <t>CAND_0057563</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>0.5207000000000001</v>
+        <v>0.8761</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Senior Data Scientist with 6.6 yrs; 6 AI core skills; response rate 0.57.</t>
+          <t>NLP Engineer with 6.8 yrs; 5 AI core skills; response rate 0.83.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CAND_0008517</t>
+          <t>CAND_0094759</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>0.5207000000000001</v>
+        <v>0.8758</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 5.6 yrs; 4 AI core skills; response rate 0.80.</t>
+          <t>Lead AI Engineer with 8.6 yrs; 8 AI core skills; response rate 0.11.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CAND_0081321</t>
+          <t>CAND_0026532</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>0.5207000000000001</v>
+        <v>0.8754</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 5.3 yrs; 4 AI core skills; response rate 0.47.</t>
+          <t>Recommendation Systems Engineer with 4.8 yrs; 6 AI core skills; response rate 0.52.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CAND_0087766</t>
+          <t>CAND_0007412</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>0.5199</v>
+        <v>0.8751</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 5.1 yrs; 6 AI core skills; response rate 0.33.</t>
+          <t>Applied ML Engineer with 7.4 yrs; 6 AI core skills; response rate 0.76.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CAND_0016170</t>
+          <t>CAND_0007009</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>0.5174</v>
+        <v>0.8742</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>AI Research Engineer with 6.8 yrs; 2 AI core skills; response rate 0.52.</t>
+          <t>Recommendation Systems Engineer with 7.9 yrs; 6 AI core skills; response rate 0.62.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CAND_0066713</t>
+          <t>CAND_0074621</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>0.5165</v>
+        <v>0.8737</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (ML) with 5.7 yrs; 2 AI core skills; response rate 0.45.</t>
+          <t>Data Scientist with 5.2 yrs; 4 AI core skills; response rate 0.74.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CAND_0050876</t>
+          <t>CAND_0044883</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>0.5145999999999999</v>
+        <v>0.8733</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Applied ML Engineer with 6.0 yrs; 6 AI core skills; response rate 0.67.</t>
+          <t>AI Engineer with 6.3 yrs; 6 AI core skills; response rate 0.84.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0033749</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>0.5121</v>
+        <v>0.8706</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer with 6.1 yrs; 5 AI core skills; response rate 0.88.</t>
+          <t>Computer Vision Engineer with 4.7 yrs; 8 AI core skills; response rate 0.78.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CAND_0077296</t>
+          <t>CAND_0000273</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>0.5087</v>
+        <v>0.8704</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Computer Vision Engineer with 5.8 yrs; 3 AI core skills; response rate 0.50.</t>
+          <t>ML Engineer with 5.8 yrs; 3 AI core skills; response rate 0.47.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CAND_0086022</t>
+          <t>CAND_0092255</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>0.5062</v>
+        <v>0.8702</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist with 5.3 yrs; 8 AI core skills; response rate 0.55.</t>
+          <t>ML Engineer with 5.2 yrs; 8 AI core skills; response rate 0.38.</t>
         </is>
       </c>
     </row>

</xml_diff>